<commit_message>
change notations in IQM harmonisation method appendix
</commit_message>
<xml_diff>
--- a/manuscript_materials/supplementary.xlsx
+++ b/manuscript_materials/supplementary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/psyc1586_admin/Desktop/harmonisation_paper/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/psyc1586_admin/GVB_data/harmonisation_work/00_aa_skullImprovement_Oct2025/00_running_for_paper/00_code_toShare/Harmonisation-Paper/manuscript_materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C45F3A6F-A4CB-4148-AB50-715AD5DD1A0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08C8CC5-ACAC-C341-B17B-82195A6A76EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17740" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17680" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="within_subject_variability" sheetId="1" r:id="rId1"/>
@@ -18356,7 +18356,7 @@
       <c r="E1" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>250</v>
       </c>
     </row>

</xml_diff>